<commit_message>
Variante 3ch: BOM Farnell corretta e snellita, progetto KiCad in zip
- LT1636: il codice 4020771 era la versione MSOP (CMS8): ora per MPN LT1636CS8#PBF
- 1N4148: 3606680 era una bobina da 5000 pezzi (24 settimane) -> 2889103 a pezzi
- test point con pin di strip header al posto dei Keystone (niente spedizione dagli USA)
- scorte MAX961/LT1636 da 17 a 16
- riv_cosmici_3ch_kicad.zip: .kicad_pro/.kicad_sch/.kicad_pcb + librerie

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/variante_3ch/BOM_farnell.xlsx
+++ b/hardware/variante_3ch/BOM_farnell.xlsx
@@ -413,14 +413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LT3461ES6#TRMPBF</t>
+          <t>LT3461AES6#TRMPBF</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -471,7 +471,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>U1 boost</t>
+          <t>U1 alta tensione (versione A, come INFN)</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -501,13 +501,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4020771</t>
-        </is>
-      </c>
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -521,16 +517,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>U?08 op-amp</t>
+          <t>U?08 op-amp - SOLO SO-8 (CS8), non MSOP (CMS8)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1685681</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="n">
         <v>12</v>
       </c>
@@ -546,14 +538,14 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>U5 U7 LDO 3.6V</t>
+          <t>U5 U7 LDO 3.6V SOT-23-5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3606680</t>
+          <t>2889103</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -561,115 +553,86 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>1N4148-TAP</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>D?01</t>
+          <t>D?01 (a pezzi, non bobina da 5000)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2250281</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="n">
-        <v>110</v>
+        <v>5</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5000</t>
+          <t>61304011121</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Keystone</t>
+          <t>Wurth Elektronik</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>test point rosso</t>
+          <t>strip 1x40 2.54 mm: header + test point</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2301278</t>
+          <t>2834673</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5001</t>
+          <t>MC-2228CG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Keystone</t>
+          <t>Multicomp</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>test point nero GND</t>
+          <t>jumper JP1-3</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2834673</t>
+          <t>4351470</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MC-2228CG</t>
+          <t>AFBR-S4N22P014M</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Multicomp</t>
+          <t>Broadcom</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
-        <is>
-          <t>jumper JP1-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>4351470</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>15</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>AFBR-S4N22P014M</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Broadcom</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
         <is>
           <t>SiPM</t>
         </is>

</xml_diff>